<commit_message>
Update Navbar with dynamic language switcher (English Version / বাংলা ভার্সন) and update Bangla Home page
</commit_message>
<xml_diff>
--- a/public/fcl-thrillers.xlsx
+++ b/public/fcl-thrillers.xlsx
@@ -100,9 +100,6 @@
     <t>Facebook Super Cup Season-02 | Match 31: Fortune Strikers vs Fearless Knight</t>
   </si>
   <si>
-    <t>https://www.facebook.com/groups/352771578172232/</t>
-  </si>
-  <si>
     <t>🔥 ৯১ রানের লক্ষ্য—কিন্তু ম্যাচ শেষ হতে লাগল মাত্র ২৩ বল!
 👑 একাই পুরো ম্যাচের নিয়ন্ত্রণ নিয়ে নিলেন Md Siyam Islam! কোনো উইকেট না হারিয়ে এমন বিধ্বংসী জয়—প্রতিপক্ষের বোলারদের জন্য ছিল এক দুঃস্বপ্নের রাত!
 😱 কীভাবে মাত্র ২৩ বলেই লেখা হলো এই অবিশ্বাস্য জয়ের গল্প?
@@ -144,15 +141,26 @@
 📖 পুরো ম্যাচের রোমাঞ্চকর গল্প জানতে ঘুরে আসুন FCL গ্রুপের মূল পোস্টে!
 🔗 https://www.facebook.com/share/p/1AMnmAeQ1X/</t>
   </si>
+  <si>
+    <t>https://www.facebook.com/share/p/17ZVwt7nev/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -175,10 +183,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -187,8 +196,10 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -543,13 +554,16 @@
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
         <v>23</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -589,36 +603,36 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="3">
         <v>41556</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3">
         <v>41465</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update rankings page layout with full-width All Players button and 3x3 role filters
</commit_message>
<xml_diff>
--- a/public/fcl-thrillers.xlsx
+++ b/public/fcl-thrillers.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Match Title</t>
   </si>
@@ -143,6 +143,27 @@
   </si>
   <si>
     <t>https://www.facebook.com/share/p/17ZVwt7nev/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1EXj4GseqA/</t>
+  </si>
+  <si>
+    <t>Sheikh Helal Ahmed</t>
+  </si>
+  <si>
+    <t>21 Balls, 91 Runs — The Run Chase Machine!</t>
+  </si>
+  <si>
+    <t>Facebook Friends Cup Season 2 — Match 29</t>
+  </si>
+  <si>
+    <t>🔥 মাত্র ২১ বলে অপরাজিত ৯১ রান! Sheikh Helal Ahmed-এর ব্যাটিং তাণ্ডবে ৯০ রানের লক্ষ্য হয়ে গেল একেবারেই তুচ্ছ!
+💥 ৭টি চার ও ৭টি ছক্কায় মাত্র ১৪টি বাউন্ডারিতেই তুলে নেন ৭০ রান। বাকি রানগুলোও আসে দুর্দান্ত গতিতে!
+⚡ FACEBOOK FRIENDS CUP Season 2-এর ২৯ নম্বর ম্যাচে Leading Stars মাত্র ৩.৩ ওভারেই, কোনো উইকেট না হারিয়ে জয় নিশ্চিত করে!
+🏆 ম্যাচসেরা Sheikh Helal Ahmed-এর এই অবিশ্বাস্য ইনিংসই তাঁকে করে তোলে EXTRA ORDINARY PERFORMANCE-এর চতুর্থ পর্বের নায়ক।
+📖 এমন বিধ্বংসী ইনিংসের পুরো গল্প জানতে ঘুরে আসুন FCL-এর মূল পোস্টে!
+🔗 https://www.facebook.com/share/p/1EXj4GseqA/
+🏏 FCL — Unity Through Cricket!</t>
   </si>
 </sst>
 </file>
@@ -478,11 +499,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="47.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" customWidth="1"/>
     <col min="3" max="3" width="45.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.140625" customWidth="1"/>
     <col min="5" max="5" width="49.42578125" bestFit="1" customWidth="1"/>
@@ -558,6 +579,23 @@
       </c>
       <c r="E4" s="4" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update extraordinary performance page with Part and Match Year badges and sorting
</commit_message>
<xml_diff>
--- a/public/fcl-thrillers.xlsx
+++ b/public/fcl-thrillers.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>Match Title</t>
   </si>
@@ -164,6 +164,32 @@
 📖 এমন বিধ্বংসী ইনিংসের পুরো গল্প জানতে ঘুরে আসুন FCL-এর মূল পোস্টে!
 🔗 https://www.facebook.com/share/p/1EXj4GseqA/
 🏏 FCL — Unity Through Cricket!</t>
+  </si>
+  <si>
+    <t>Ovi Raihan Remembrance Special Series 2025 — Match 15</t>
+  </si>
+  <si>
+    <t>Zaheed Hasan &amp; Sumon AB</t>
+  </si>
+  <si>
+    <t>Match-Winning All-Round Performance &amp; Explosive Batting</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1BjuJcExb2/</t>
+  </si>
+  <si>
+    <t>🔥 একদিকে Sumon AB-এর ১৬ বলে বিধ্বংসী ৫৯ রান, অন্যদিকে Zaheed Hasan-এর বল হাতে ৩ উইকেট ও ব্যাট হাতে ১০ বলে অপরাজিত ৩৮ রানের ম্যাচজয়ী পারফরম্যান্স!
+⚡ মাত্র ৫ রানে ৩ উইকেট হারিয়েও Sumon AB-এর ব্যাটিং ঝড়ে OVI RAIHAN TITANS তুলে নেয় ৯৭ রান।
+💥 কিন্তু ৯৮ রানের লক্ষ্য তাড়া করতে নেমে শেষ পর্যন্ত জয়ের নায়ক হয়ে ওঠেন Zaheed Hasan! তাঁর অপরাজিত ইনিংসে ৩ উইকেটের জয় নিশ্চিত করে OVI RAIHAN PHOENIX।
+🏆 OVI RAIHAN REMEMBRANCE SPECIAL SERIES 2025-এর ১৫ নম্বর ম্যাচে একজন গড়েছিলেন লড়াইয়ের মঞ্চ, আর অন্যজন ছিনিয়ে নেন জয়!
+🌟 ম্যাচসেরা Zaheed Hasan, আর CPOM Sumon AB — দুই অসাধারণ পারফরম্যান্সের এক রোমাঞ্চকর গল্প!
+🏏 FCL — Unity Through Cricket!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part </t>
+  </si>
+  <si>
+    <t>Match Year</t>
   </si>
 </sst>
 </file>
@@ -208,7 +234,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -218,6 +244,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -499,108 +526,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.7109375" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="49.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="54.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="68.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="49.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2016</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2016</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2020</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2020</v>
+      </c>
+      <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1"/>
+    <hyperlink ref="G4" r:id="rId1"/>
+    <hyperlink ref="G6" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix layout overlap in PlayerCardModal and update component
</commit_message>
<xml_diff>
--- a/public/fcl-thrillers.xlsx
+++ b/public/fcl-thrillers.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Extraordinary Performance" sheetId="1" r:id="rId1"/>
@@ -686,6 +686,7 @@
     <hyperlink ref="G6" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -758,5 +759,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>